<commit_message>
Added Integration Test - two new classes: EmploymentStatistics.java and HealthStatistics.java - provide additional statistics necessary for Integration test - details on Integration test are described in README.md of integrationtest/expected folder - fixed PartnershipAlignment to stop mutating shared matching pools from a parallelStream() - it now calls a simple sequential helper.
</commit_message>
<xml_diff>
--- a/input/DatabaseCountryYear.xlsx
+++ b/input/DatabaseCountryYear.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="6">
   <si>
     <t>Country</t>
   </si>
@@ -24,6 +24,12 @@
   </si>
   <si>
     <t>2011</t>
+  </si>
+  <si>
+    <t>2013</t>
+  </si>
+  <si>
+    <t>2019</t>
   </si>
 </sst>
 </file>
@@ -84,7 +90,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- optimized singlerun to reuse input.mv.db if it exists; - to force rebuild of input.mv.db - set reuseExistingDatabase = false or use the follwoing commmands: "java -jar singlerun.jar -c PL -s 2011 -g false -Setup" "java -jar singlerun.jar -c PL -s 2011 -g false --rebuild-db" - also, SimPathsEU should run well for PL even when InitialPopulations or EUROMODoutput data are missing for other countries - updated README.md
</commit_message>
<xml_diff>
--- a/input/DatabaseCountryYear.xlsx
+++ b/input/DatabaseCountryYear.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="6">
   <si>
     <t>Country</t>
   </si>
@@ -90,7 +90,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated CLAUDE.md and other supporting files
</commit_message>
<xml_diff>
--- a/input/DatabaseCountryYear.xlsx
+++ b/input/DatabaseCountryYear.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="9">
   <si>
     <t>Country</t>
   </si>
@@ -30,6 +30,15 @@
   </si>
   <si>
     <t>2019</t>
+  </si>
+  <si>
+    <t>ES</t>
+  </si>
+  <si>
+    <t>2017</t>
+  </si>
+  <si>
+    <t>2022</t>
   </si>
 </sst>
 </file>
@@ -87,10 +96,10 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: allow simulation start years up to 2023
`Parameters.MAX_START_YEAR` was 2020, which is the guard on how recent an
initial population a run may start from. The Polish initial population and
its parameter tables now extend to 2023, so the guard was rejecting start
years the input data actually supports.

Raised the ceiling to 2023 and updated the two workbooks that have to agree
with it:

- `input/DatabaseCountryYear.xlsx` — the country/year table the database
  setup reads to decide which initial population to build.
- `input/PL/parameters.xlsx` — the PL parameter tables, extended over the
  same span.

`MIN_START_YEAR` is untouched, so every previously valid start year stays
valid; this only widens the accepted range.
</commit_message>
<xml_diff>
--- a/input/DatabaseCountryYear.xlsx
+++ b/input/DatabaseCountryYear.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="8">
   <si>
     <t>Country</t>
   </si>
@@ -30,6 +30,12 @@
   </si>
   <si>
     <t>2019</t>
+  </si>
+  <si>
+    <t>2020</t>
+  </si>
+  <si>
+    <t>2023</t>
   </si>
 </sst>
 </file>
@@ -90,7 +96,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>